<commit_message>
Add grant-advisor orchestration skill (URL/PDF to decision to tracker to folder); align decision labels; reset tracker
</commit_message>
<xml_diff>
--- a/grants/grant-tracker.xlsx
+++ b/grants/grant-tracker.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -426,7 +426,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
@@ -490,63 +490,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NSF HBCU Excellence in Research (HBCU-EiR)</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>National Science Foundation</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>HBCU-EiR</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>See current NOFO</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>up to ~$500K / 3 yrs</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Go</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Reviewing</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>grants/EXAMPLE-NSF-HBCU-EiR/</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Worked example; delete with the EXAMPLE- folder.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hybrid tracker: Gosha ops columns + AI eval columns, dropdowns, drop Folder; grant-organizer matches on Name and preserves researcher-entered fields
</commit_message>
<xml_diff>
--- a/grants/grant-tracker.xlsx
+++ b/grants/grant-tracker.xlsx
@@ -417,80 +417,136 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Grant / Opportunity</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Funder</t>
+          <t>Agency</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Program / Opportunity #</t>
+          <t>Program</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Deadline</t>
+          <t>Website</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Award Range</t>
+          <t>I'm PI?</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Co-PIs / Lead</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>LOI Date</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Route By</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Target Submit</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Routed?</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Previously Submitted?</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Fit Rating</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Date Reviewed</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Folder</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="6">
+    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Strong,Moderate,Weak,Not eligible"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pursue,Considering,Don't Pursue"</formula1>
+    </dataValidation>
+    <dataValidation sqref="P2:P500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Reviewing,Drafting,Submitted,Awarded,Declined"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
NSF refactor: rename grant-writing to nsf-grant-writer; split out grant-review; retire nsf-broader-impacts (folded into references); NSF sections + 10 grant types
</commit_message>
<xml_diff>
--- a/grants/grant-tracker.xlsx
+++ b/grants/grant-tracker.xlsx
@@ -1,40 +1,114 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ashleyscruse/Documents/scruse-hq/03 workspaces/ashleyscruse-com/grant-writing-starter/grants/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DBE2510-CFA5-C54D-82DA-6CB803C26EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grants" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Grants" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Agency</t>
+  </si>
+  <si>
+    <t>Program</t>
+  </si>
+  <si>
+    <t>Website</t>
+  </si>
+  <si>
+    <t>I'm PI?</t>
+  </si>
+  <si>
+    <t>Co-PIs / Lead</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>LOI Date</t>
+  </si>
+  <si>
+    <t>Due Date</t>
+  </si>
+  <si>
+    <t>Route By</t>
+  </si>
+  <si>
+    <t>Target Submit</t>
+  </si>
+  <si>
+    <t>Routed?</t>
+  </si>
+  <si>
+    <t>Previously Submitted?</t>
+  </si>
+  <si>
+    <t>Fit Rating</t>
+  </si>
+  <si>
+    <t>Decision</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri (Body)"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri (Body)"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,82 +123,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -412,138 +428,92 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="40" customWidth="1" min="17" max="17"/>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="30" customWidth="1"/>
+    <col min="5" max="5" width="9" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="13" customWidth="1"/>
+    <col min="12" max="12" width="9" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="16" customWidth="1"/>
+    <col min="16" max="16" width="12" customWidth="1"/>
+    <col min="17" max="17" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Agency</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Program</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>I'm PI?</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Co-PIs / Lead</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>LOI Date</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Route By</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Target Submit</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Routed?</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Previously Submitted?</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Fit Rating</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Decision</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
+    <row r="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" sqref="E2:E500 L2:M500" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No"</formula1>
-    </dataValidation>
-    <dataValidation sqref="M2:M500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No"</formula1>
-    </dataValidation>
-    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation type="list" allowBlank="1" sqref="N2:N500" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Strong,Moderate,Weak,Not eligible"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation type="list" allowBlank="1" sqref="O2:O500" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Pursue,Considering,Don't Pursue"</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation type="list" allowBlank="1" sqref="P2:P500" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Reviewing,Drafting,Submitted,Awarded,Declined"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>